<commit_message>
Update source docs (corrected Cert III F2F/VOF) as new standard; trim now-redundant adjustments
</commit_message>
<xml_diff>
--- a/output/normalised.xlsx
+++ b/output/normalised.xlsx
@@ -5979,7 +5979,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Graham Barber</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -6066,12 +6066,12 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">21/07/2026 01/12/2026</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Graham Barber</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -6531,7 +6531,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jennie Agustin</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -6715,7 +6715,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Anu Joshi</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Graham Barber; Graham Barber; Anu Joshi</t>
+          <t xml:space="preserve">Graham Barber</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -7150,12 +7150,12 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTCLD301 Evaluate Characteristics of Cloud Computing solutions and services | ICTICT310 Identify and use industry specific technologies.</t>
+          <t xml:space="preserve">ICTCLD301 Evaluate Characteristics of Cloud Computing solutions and services</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTCLD301, ICTICT310</t>
+          <t xml:space="preserve">ICTCLD301</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -7165,17 +7165,17 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t xml:space="preserve">10-14 14-18</t>
+          <t xml:space="preserve">10-14</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t xml:space="preserve">24/09/2026 29/10/2026 5/11/2026 03/12/202</t>
+          <t xml:space="preserve">24/09/2026 29/10/2026</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Graham Barber</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -7197,17 +7197,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICT40120 Cert IV  Programming OUR.docx</t>
+          <t xml:space="preserve">ICT30120 Cert III General VOF OUR.docx</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cert IV Programming</t>
+          <t xml:space="preserve">Cert III General (VOFF)</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICT40120</t>
+          <t xml:space="preserve">ICT30120</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7217,12 +7217,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monday</t>
+          <t xml:space="preserve">Thursday</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t xml:space="preserve">1a Mon 1b Mon</t>
+          <t xml:space="preserve">3A Thu 3B Thu 3C Thu</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -7232,7 +7232,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t xml:space="preserve">12:00</t>
+          <t xml:space="preserve">2:30</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -7242,37 +7242,37 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSBXCS404 Contribute to cyber security risk management. | ICTICT443 Work collaboratively in the ICT industry | ICTICT451 Comply with IP, ethics and privacy policies in ICT environments</t>
+          <t xml:space="preserve">ICTICT310 Identify and use industry specific technologies.</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSBXCS404, ICTICT443, ICTICT451</t>
+          <t xml:space="preserve">ICTICT310</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Graham on Campus</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t xml:space="preserve">1-8</t>
+          <t xml:space="preserve">14-18</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t xml:space="preserve">20/07/2026 7/09/2026</t>
+          <t xml:space="preserve">5/11/2026 03/12/202</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Graham Barber and; Rima Andrews</t>
+          <t xml:space="preserve">Anu Joshi</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t xml:space="preserve">F2F</t>
+          <t xml:space="preserve">VOFF</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -7282,7 +7282,7 @@
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
     </row>
@@ -7334,12 +7334,12 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSBCRT404 Apply advanced critical thinking to work processes | ICTICT426 Identify and evaluate emerging technologies and practices | ICTSAS432 Identify and resolve client ICT problems</t>
+          <t xml:space="preserve">BSBXCS404 Contribute to cyber security risk management. | ICTICT443 Work collaboratively in the ICT industry | ICTICT451 Comply with IP, ethics and privacy policies in ICT environments</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSBCRT404, ICTICT426, ICTSAS432</t>
+          <t xml:space="preserve">BSBXCS404, ICTICT443, ICTICT451</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -7349,17 +7349,17 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t xml:space="preserve">9-18</t>
+          <t xml:space="preserve">1-8</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t xml:space="preserve">14/09/2026 30/11/2026</t>
+          <t xml:space="preserve">20/07/2026 7/09/2026</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Graham Barber</t>
+          <t xml:space="preserve">Graham Barber and; Rima Andrews</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
     </row>
@@ -7401,12 +7401,12 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tuesday</t>
+          <t xml:space="preserve">Monday</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t xml:space="preserve">2a Tue 2b Tue 2c Tue 2d Tue</t>
+          <t xml:space="preserve">1a Mon 1b Mon</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -7416,47 +7416,47 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t xml:space="preserve">10:00</t>
+          <t xml:space="preserve">12:00</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tutorial Support</t>
+          <t xml:space="preserve">Teaching</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">BSBCRT404 Apply advanced critical thinking to work processes | ICTICT426 Identify and evaluate emerging technologies and practices | ICTSAS432 Identify and resolve client ICT problems</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">BSBCRT404, ICTICT426, ICTSAS432</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tutorial Support | Shanna on Campus</t>
+          <t xml:space="preserve">Graham on Campus</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t xml:space="preserve">1-18</t>
+          <t xml:space="preserve">9-18</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">14/09/2026 30/11/2026</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shaun Stummer Online; Shanna Roper F2F</t>
+          <t xml:space="preserve">Graham Barber</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t xml:space="preserve">F2F/VOFF</t>
+          <t xml:space="preserve">F2F</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -7466,7 +7466,7 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
     </row>
@@ -7503,52 +7503,52 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
+          <t xml:space="preserve">9:00</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
           <t xml:space="preserve">10:00</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3:30</t>
-        </is>
-      </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teaching</t>
+          <t xml:space="preserve">Tutorial Support</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTPRG440 Apply introductory programming skills in different languages | ICTWEB431 Create and style simple markup language</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTPRG440, ICTWEB431</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Different assessments | Shanna on Campus</t>
+          <t xml:space="preserve">Tutorial Support | Shanna on Campus</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t xml:space="preserve">1-11</t>
+          <t xml:space="preserve">1-18</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t xml:space="preserve">21/07/2026 13/10/2026</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shaun Stummer; Shanna Roper</t>
+          <t xml:space="preserve">Shaun Stummer Online; Shanna Roper F2F</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t xml:space="preserve">F2F</t>
+          <t xml:space="preserve">F2F/VOFF</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
     </row>
@@ -7610,37 +7610,37 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTPRG441 Apply skills in object-oriented design | ICTPRG444 Analyse software requirements</t>
+          <t xml:space="preserve">ICTPRG440 Apply introductory programming skills in different languages | ICTWEB431 Create and style simple markup language</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTPRG441, ICTPRG444</t>
+          <t xml:space="preserve">ICTPRG440, ICTWEB431</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Different assessments | Shanna on Campus</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t xml:space="preserve">12-18</t>
+          <t xml:space="preserve">1-11</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t xml:space="preserve">20/10/2026 3/12/2026</t>
+          <t xml:space="preserve">21/07/2026 13/10/2026</t>
         </is>
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shaun Stummer</t>
+          <t xml:space="preserve">Shaun Stummer; Shanna Roper</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">F2F</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -7650,7 +7650,7 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
     </row>
@@ -7677,17 +7677,17 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wednesday</t>
+          <t xml:space="preserve">Tuesday</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t xml:space="preserve">3a Wed 3b Wed</t>
+          <t xml:space="preserve">2a Tue 2b Tue 2c Tue 2d Tue</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t xml:space="preserve">9:00</t>
+          <t xml:space="preserve">10:00</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -7702,12 +7702,12 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTDBS416 Create basic relational databases | ICTPRG431 Apply query language in relational databases</t>
+          <t xml:space="preserve">ICTPRG441 Apply skills in object-oriented design | ICTPRG444 Analyse software requirements</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTDBS416, ICTPRG431</t>
+          <t xml:space="preserve">ICTPRG441, ICTPRG444</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -7717,17 +7717,17 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t xml:space="preserve">1-8</t>
+          <t xml:space="preserve">12-18</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t xml:space="preserve">22/07/2026 09/09/2026</t>
+          <t xml:space="preserve">20/10/2026 3/12/2026</t>
         </is>
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shaun Stummer and Anu Joshi</t>
+          <t xml:space="preserve">Shaun Stummer</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
@@ -7742,7 +7742,7 @@
       </c>
       <c r="R84" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
     </row>
@@ -7794,12 +7794,12 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTPRG436 Develop mobile applications | ICTPRG437 Build a user interface | ICTICT449 Use version control systems in development environment</t>
+          <t xml:space="preserve">ICTDBS416 Create basic relational databases | ICTPRG431 Apply query language in relational databases</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTPRG436, ICTPRG437, ICTICT449</t>
+          <t xml:space="preserve">ICTDBS416, ICTPRG431</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -7809,12 +7809,12 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t xml:space="preserve">9-18</t>
+          <t xml:space="preserve">1-8</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t xml:space="preserve">16/09/2026 2/12/2026</t>
+          <t xml:space="preserve">22/07/2026 09/09/2026</t>
         </is>
       </c>
       <c r="O85" t="inlineStr">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
     </row>
@@ -7861,70 +7861,162 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
+          <t xml:space="preserve">Wednesday</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3a Wed 3b Wed</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9:00</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3:30</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teaching</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICTPRG436 Develop mobile applications | ICTPRG437 Build a user interface | ICTICT449 Use version control systems in development environment</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICTPRG436, ICTPRG437, ICTICT449</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9-18</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16/09/2026 2/12/2026</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shaun Stummer and Anu Joshi</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICT40120 Cert IV  Programming OUR.docx</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cert IV Programming</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICT40120</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2 2026</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
           <t xml:space="preserve">Thursday</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F87" t="inlineStr">
         <is>
           <t xml:space="preserve">4a Thu</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
+      <c r="G87" t="inlineStr">
         <is>
           <t xml:space="preserve">9:00</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="H87" t="inlineStr">
         <is>
           <t xml:space="preserve">3:30</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr">
+      <c r="I87" t="inlineStr">
         <is>
           <t xml:space="preserve">Teaching</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr">
+      <c r="J87" t="inlineStr">
         <is>
           <t xml:space="preserve">ICTPRG302 Apply introductory programming techniques | ICTPRG432 Develop data driven Apps | ICTPRG439 Use pre-existing components | ICTPRG430 Apply introductory object-oriented language skills | ICTPRG433 Test software developments</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr">
+      <c r="K87" t="inlineStr">
         <is>
           <t xml:space="preserve">ICTPRG302, ICTPRG432, ICTPRG439, ICTPRG430, ICTPRG433</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="M86" t="inlineStr">
+      <c r="L87" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
         <is>
           <t xml:space="preserve">1-18</t>
         </is>
       </c>
-      <c r="N86" t="inlineStr">
+      <c r="N87" t="inlineStr">
         <is>
           <t xml:space="preserve">23/07/2026 3/12/2026</t>
         </is>
       </c>
-      <c r="O86" t="inlineStr">
+      <c r="O87" t="inlineStr">
         <is>
           <t xml:space="preserve">Shaun Stummer and  Anu Joshi</t>
         </is>
       </c>
-      <c r="P86" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Q86" t="inlineStr">
+      <c r="P87" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="R86" t="inlineStr">
+      <c r="R87" t="inlineStr">
         <is>
           <t xml:space="preserve">8</t>
         </is>
@@ -8194,7 +8286,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Graham Barber</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -8281,12 +8373,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">21/07/2026 01/12/2026</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Graham Barber</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -8746,7 +8838,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jennie Agustin</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -9029,7 +9121,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Anu Joshi</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -9397,7 +9489,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Graham Barber; Graham Barber; Anu Joshi</t>
+          <t xml:space="preserve">Graham Barber</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -9464,12 +9556,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTCLD301 Evaluate Characteristics of Cloud Computing solutions and services | ICTICT310 Identify and use industry specific technologies.</t>
+          <t xml:space="preserve">ICTCLD301 Evaluate Characteristics of Cloud Computing solutions and services</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICTCLD301, ICTICT310</t>
+          <t xml:space="preserve">ICTCLD301</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -9479,17 +9571,17 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t xml:space="preserve">10-14 14-18</t>
+          <t xml:space="preserve">10-14</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t xml:space="preserve">24/09/2026 29/10/2026 5/11/2026 03/12/202</t>
+          <t xml:space="preserve">24/09/2026 29/10/2026</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Graham Barber</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -9505,6 +9597,98 @@
       <c r="R8" t="inlineStr">
         <is>
           <t xml:space="preserve">7</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICT30120 Cert III General VOF OUR.docx</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cert III General (VOFF)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICT30120</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2 2026</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thursday</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3A Thu 3B Thu 3C Thu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9:00</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2:30</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teaching</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICTICT310 Identify and use industry specific technologies.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICTICT310</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14-18</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5/11/2026 03/12/202</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anu Joshi</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VOFF</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
     </row>
@@ -16538,116 +16722,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NEEDS-TEACHER</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ICT30120 Cert III  General F2F OUR.docx</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cert III General (F2F)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Cert III General (F2F)] Tuesday 9:00-2:30 'ICTCLD301 Evaluate Characteristics of Cloud Computing Solutions and services. | BSBXCS303 Securely manage personally identifiable information and workplace information. | ICTICT313 Identify IP, ethics, and privacy policies in ICT environments.' has NO teacher.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NEEDS-TEACHER</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ICT30120 Cert III  General F2F OUR.docx</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cert III General (F2F)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Cert III General (F2F)] Tuesday 2:30-3:30 'Tutorial Support' has NO teacher.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NEEDS-TEACHER</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ICT30120 Cert III  General F2F OUR.docx</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cert III General (F2F)</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Cert III General (F2F)] Thursday 9:00-2:30 'ICTPRG302 Apply introductory programming techniques.' has NO teacher.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NEEDS-TEACHER</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ICT30120 Cert III General VOF OUR.docx</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cert III General (VOFF)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Cert III General (VOFF)] Tuesday 9:00-2:30 'BSBCRT301 Develop and extend critical and creative thinking skills. | BSBXTW301 Work in a team. | ICTSAS305 Provide ICT advice to clients.' has NO teacher.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NEEDS-TEACHER</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ICT30120 Cert III General VOF OUR.docx</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cert III General (VOFF)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Cert III General (VOFF)] Thursday 9:00-2:30 'ICTCLD301 Evaluate Characteristics of Cloud Computing solutions and services | ICTICT310 Identify and use industry specific technologies.' has NO teacher.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>